<commit_message>
feat(functions): add backend safety audit-wave foundations (hb-intel-safety 1.2.11.0 unchanged)
Register the safety record-keeping admin routes in the monolithic functions host, extend the legacy-fallback Graph list client with list-existence and writable-column discovery helpers, and add the backend phase-01 audit/wave planning package plus the updated Safety checklist template artifact. Safety SPFx manifest title/version remain HB Intel Safety / 1.2.11.0 in this commit.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/architecture/plans/MASTER/spfx/safety-records/Safety Checklist Template.xlsx
+++ b/docs/architecture/plans/MASTER/spfx/safety-records/Safety Checklist Template.xlsx
@@ -5,22 +5,41 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bobbyfetting/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bobbyfetting/hb-intel/docs/architecture/plans/MASTER/spfx/safety-records/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DCBAA39-A508-FD43-A906-6C8B3AC3CF76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{623ABEA3-9CAA-B147-A3B9-A93B1377E785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="660" windowWidth="24720" windowHeight="17440" xr2:uid="{6F937327-2405-48D2-A075-7D7A02836D6F}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="30240" windowHeight="19460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScoreCard" sheetId="1" r:id="rId1"/>
     <sheet name="ScoringWeights" sheetId="2" r:id="rId2"/>
+    <sheet name="ParserMeta" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <definedNames>
+    <definedName name="InspectionDateCell">ScoreCard!$B$3</definedName>
+    <definedName name="InspectionNumberCell">ScoreCard!$E$3</definedName>
+    <definedName name="KeyFindingsLines">ScoreCard!$A$143:$A$148</definedName>
+    <definedName name="KeyFindingsVisualBlock">ScoreCard!$A$143:$G$148</definedName>
+    <definedName name="ParserContractVersion">ParserMeta!$B$3</definedName>
+    <definedName name="ParserInspectionDateRaw">ParserMeta!$B$4</definedName>
+    <definedName name="ParserInspectionNumberRaw">ParserMeta!$B$5</definedName>
+    <definedName name="ParserKeyFindingsNormalized">ParserMeta!$B$14</definedName>
+    <definedName name="ParserProjectSiteRaw">ParserMeta!$B$6</definedName>
+    <definedName name="ParserReportingPeriodLabel">ParserMeta!$B$13</definedName>
+    <definedName name="ParserReportingWeekEnd">ParserMeta!$B$12</definedName>
+    <definedName name="ParserReportingWeekStart">ParserMeta!$B$11</definedName>
+    <definedName name="ParserTemplateVersion">ParserMeta!$B$2</definedName>
+    <definedName name="ProjectSiteCell">ScoreCard!$B$4</definedName>
+    <definedName name="SafetyScoreCell">ScoreCard!$G$7</definedName>
+    <definedName name="TotalNACell">ScoreCard!$G$6</definedName>
+    <definedName name="TotalNoCell">ScoreCard!$G$5</definedName>
+    <definedName name="TotalYesCell">ScoreCard!$G$4</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -59,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="173">
   <si>
     <t>Construction Site Safety Walk Checklist (Field Form)</t>
   </si>
@@ -485,102 +504,177 @@
   </si>
   <si>
     <t>Total Weight Allocation:</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>TemplateVersion</t>
+  </si>
+  <si>
+    <t>SafetyChecklist_v1</t>
+  </si>
+  <si>
+    <t>Explicit template/version marker for downstream parsing.</t>
+  </si>
+  <si>
+    <t>ParserContractVersion</t>
+  </si>
+  <si>
+    <t>parse-first-2026-04</t>
+  </si>
+  <si>
+    <t>Workbook-side parser contract revision.</t>
+  </si>
+  <si>
+    <t>InspectionDateRaw</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!B3.</t>
+  </si>
+  <si>
+    <t>InspectionNumberRaw</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!E3.</t>
+  </si>
+  <si>
+    <t>ProjectSiteRaw</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!B4.</t>
+  </si>
+  <si>
+    <t>TotalYes</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!G4.</t>
+  </si>
+  <si>
+    <t>TotalNo</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!G5.</t>
+  </si>
+  <si>
+    <t>TotalNA</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!G6.</t>
+  </si>
+  <si>
+    <t>SafetyScore</t>
+  </si>
+  <si>
+    <t>Direct mirror of ScoreCard!G7.</t>
+  </si>
+  <si>
+    <t>ReportingWeekStart</t>
+  </si>
+  <si>
+    <t>Derived Monday date from the inspection date.</t>
+  </si>
+  <si>
+    <t>ReportingWeekEnd</t>
+  </si>
+  <si>
+    <t>Derived Friday date from the inspection date.</t>
+  </si>
+  <si>
+    <t>ReportingPeriodLabel</t>
+  </si>
+  <si>
+    <t>Readable Monday–Friday reporting-period label.</t>
+  </si>
+  <si>
+    <t>KeyFindingsNormalized</t>
+  </si>
+  <si>
+    <t>Concatenated free-text findings block from the visible worksheet.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F4E79"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -598,7 +692,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF353AF7"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -613,8 +706,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -785,7 +878,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -851,38 +944,20 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -908,23 +983,44 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="145">
+  <dxfs count="135">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -957,6 +1053,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -977,11 +1093,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -997,6 +1113,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1017,6 +1143,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1047,6 +1183,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1067,6 +1223,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1087,11 +1283,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1107,11 +1303,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1157,6 +1373,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1186,1004 +1432,662 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="13" formatCode="0%"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="13" formatCode="0%"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2199,24 +2103,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46D8C12E-7807-4B9F-A2D9-5025801EC560}" name="tblWeights" displayName="tblWeights" ref="A1:D14" totalsRowCount="1" headerRowDxfId="144" dataDxfId="143">
-  <autoFilter ref="A1:D13" xr:uid="{46D8C12E-7807-4B9F-A2D9-5025801EC560}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblWeights" displayName="tblWeights" ref="A1:D14">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3BCD8EF1-DD23-4FFF-8A10-0D15BDEC377A}" name="Num" dataDxfId="142" totalsRowDxfId="141"/>
-    <tableColumn id="2" xr3:uid="{FBAE33BE-B888-46C2-8482-0CFD86063900}" name="Section" totalsRowLabel="Total Weight Allocation:" dataDxfId="140" totalsRowDxfId="139"/>
-    <tableColumn id="3" xr3:uid="{D1EFD63C-8C1F-4A94-BC26-E61D48063F6F}" name="Weight" totalsRowFunction="custom" dataDxfId="138" totalsRowDxfId="137">
-      <totalsRowFormula>SUM(tblWeights[Weight])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{C15D1362-A246-4843-9559-EFB68FCD522C}" name="Rationale (Risk to Life / Serious Injury)" totalsRowFunction="custom" dataDxfId="136" totalsRowDxfId="135">
-      <totalsRowFormula>IF(ABS(1-SUM(tblWeights[Weight]))&lt;=0.000001,"",IF(1-SUM(tblWeights[Weight])&gt;0,"Add "&amp;TEXT(1-SUM(tblWeights[Weight]),"0%")&amp;" to the category weights","Deduct "&amp;TEXT(ABS(1-SUM(tblWeights[Weight])),"0%")&amp;" from the category weights"))</totalsRowFormula>
-    </tableColumn>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Num"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Section" totalsRowLabel="Total Weight Allocation:"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Weight"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Rationale (Risk to Life / Serious Injury)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2258,108 +2157,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -2367,80 +2172,31 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="dk1"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="accent1"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -2470,22 +2226,22 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -2500,68 +2256,13 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{F763305E-451D-4EB3-A6B4-C8C335A6BF8C}">
-  <we:reference id="WA200009404" version="1.0.0.8" store="en-us" storeType="omex"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="en-us" storeType="omex"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45333986-184E-4200-A045-50F5AEF7C1DF}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2573,38 +2274,42 @@
     <col min="7" max="7" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="39" t="s">
+    <row r="1" spans="1:9" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="42"/>
+      <c r="B3" s="37">
+        <v>46068</v>
+      </c>
+      <c r="C3" s="38"/>
       <c r="D3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="43" t="s">
+      <c r="E3" s="16">
+        <v>5</v>
+      </c>
+      <c r="F3" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="44"/>
-    </row>
-    <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G3" s="40"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="42"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="38"/>
       <c r="D4" s="17"/>
       <c r="E4" s="16"/>
       <c r="F4" s="15" t="s">
@@ -2615,10 +2320,10 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17"/>
-      <c r="B5" s="45"/>
-      <c r="C5" s="42"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="38"/>
       <c r="F5" s="15" t="s">
         <v>6</v>
       </c>
@@ -2645,7 +2350,7 @@
         <v>0.85671428571428576</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>9</v>
       </c>
@@ -2668,16 +2373,16 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36" t="s">
+    <row r="10" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="38"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="34"/>
     </row>
     <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
@@ -2883,16 +2588,16 @@
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
     </row>
-    <row r="22" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="32" t="s">
+    <row r="22" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="34"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="45"/>
     </row>
     <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
@@ -2998,16 +2703,16 @@
       <c r="F28" s="11"/>
       <c r="G28" s="11"/>
     </row>
-    <row r="29" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="32" t="s">
+    <row r="29" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="33"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="34"/>
+      <c r="B29" s="44"/>
+      <c r="C29" s="44"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="45"/>
     </row>
     <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
@@ -3171,16 +2876,16 @@
       <c r="F38" s="11"/>
       <c r="G38" s="11"/>
     </row>
-    <row r="39" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="32" t="s">
+    <row r="39" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="34"/>
+      <c r="B39" s="44"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="44"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="45"/>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
@@ -3385,16 +3090,16 @@
       <c r="F50" s="11"/>
       <c r="G50" s="11"/>
     </row>
-    <row r="51" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="32" t="s">
+    <row r="51" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="33"/>
-      <c r="C51" s="33"/>
-      <c r="D51" s="33"/>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="34"/>
+      <c r="B51" s="44"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
+      <c r="F51" s="44"/>
+      <c r="G51" s="45"/>
     </row>
     <row r="52" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
@@ -3633,16 +3338,16 @@
       <c r="F64" s="11"/>
       <c r="G64" s="11"/>
     </row>
-    <row r="65" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="32" t="s">
+    <row r="65" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="B65" s="33"/>
-      <c r="C65" s="33"/>
-      <c r="D65" s="33"/>
-      <c r="E65" s="33"/>
-      <c r="F65" s="33"/>
-      <c r="G65" s="34"/>
+      <c r="B65" s="44"/>
+      <c r="C65" s="44"/>
+      <c r="D65" s="44"/>
+      <c r="E65" s="44"/>
+      <c r="F65" s="44"/>
+      <c r="G65" s="45"/>
     </row>
     <row r="66" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="9" t="s">
@@ -3805,16 +3510,16 @@
       <c r="F74" s="11"/>
       <c r="G74" s="11"/>
     </row>
-    <row r="75" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="32" t="s">
+    <row r="75" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="B75" s="33"/>
-      <c r="C75" s="33"/>
-      <c r="D75" s="33"/>
-      <c r="E75" s="33"/>
-      <c r="F75" s="33"/>
-      <c r="G75" s="34"/>
+      <c r="B75" s="44"/>
+      <c r="C75" s="44"/>
+      <c r="D75" s="44"/>
+      <c r="E75" s="44"/>
+      <c r="F75" s="44"/>
+      <c r="G75" s="45"/>
     </row>
     <row r="76" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="9" t="s">
@@ -3939,16 +3644,16 @@
       <c r="F82" s="11"/>
       <c r="G82" s="11"/>
     </row>
-    <row r="83" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="32" t="s">
+    <row r="83" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="B83" s="33"/>
-      <c r="C83" s="33"/>
-      <c r="D83" s="33"/>
-      <c r="E83" s="33"/>
-      <c r="F83" s="33"/>
-      <c r="G83" s="34"/>
+      <c r="B83" s="44"/>
+      <c r="C83" s="44"/>
+      <c r="D83" s="44"/>
+      <c r="E83" s="44"/>
+      <c r="F83" s="44"/>
+      <c r="G83" s="45"/>
     </row>
     <row r="84" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" s="9" t="s">
@@ -4073,16 +3778,16 @@
       <c r="F90" s="11"/>
       <c r="G90" s="11"/>
     </row>
-    <row r="91" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="32" t="s">
+    <row r="91" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="43" t="s">
         <v>90</v>
       </c>
-      <c r="B91" s="33"/>
-      <c r="C91" s="33"/>
-      <c r="D91" s="33"/>
-      <c r="E91" s="33"/>
-      <c r="F91" s="33"/>
-      <c r="G91" s="34"/>
+      <c r="B91" s="44"/>
+      <c r="C91" s="44"/>
+      <c r="D91" s="44"/>
+      <c r="E91" s="44"/>
+      <c r="F91" s="44"/>
+      <c r="G91" s="45"/>
     </row>
     <row r="92" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" s="9" t="s">
@@ -4266,16 +3971,16 @@
       <c r="F101" s="10"/>
       <c r="G101" s="10"/>
     </row>
-    <row r="102" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="32" t="s">
+    <row r="102" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="B102" s="33"/>
-      <c r="C102" s="33"/>
-      <c r="D102" s="33"/>
-      <c r="E102" s="33"/>
-      <c r="F102" s="33"/>
-      <c r="G102" s="34"/>
+      <c r="B102" s="44"/>
+      <c r="C102" s="44"/>
+      <c r="D102" s="44"/>
+      <c r="E102" s="44"/>
+      <c r="F102" s="44"/>
+      <c r="G102" s="45"/>
     </row>
     <row r="103" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="9" t="s">
@@ -4400,16 +4105,16 @@
       <c r="F109" s="11"/>
       <c r="G109" s="11"/>
     </row>
-    <row r="110" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="35" t="s">
+    <row r="110" spans="1:9" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="B110" s="35"/>
-      <c r="C110" s="35"/>
-      <c r="D110" s="35"/>
-      <c r="E110" s="35"/>
-      <c r="F110" s="35"/>
-      <c r="G110" s="35"/>
+      <c r="B110" s="46"/>
+      <c r="C110" s="46"/>
+      <c r="D110" s="46"/>
+      <c r="E110" s="46"/>
+      <c r="F110" s="46"/>
+      <c r="G110" s="46"/>
     </row>
     <row r="111" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" s="9" t="s">
@@ -4553,16 +4258,16 @@
       <c r="F118" s="11"/>
       <c r="G118" s="11"/>
     </row>
-    <row r="119" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="35" t="s">
+    <row r="119" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="B119" s="35"/>
-      <c r="C119" s="35"/>
-      <c r="D119" s="35"/>
-      <c r="E119" s="35"/>
-      <c r="F119" s="35"/>
-      <c r="G119" s="35"/>
+      <c r="B119" s="46"/>
+      <c r="C119" s="46"/>
+      <c r="D119" s="46"/>
+      <c r="E119" s="46"/>
+      <c r="F119" s="46"/>
+      <c r="G119" s="46"/>
     </row>
     <row r="120" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A120" s="9" t="s">
@@ -4678,17 +4383,17 @@
       <c r="G126" s="11"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A127" s="31" t="s">
+      <c r="A127" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="B127" s="31"/>
-      <c r="C127" s="31"/>
-      <c r="D127" s="31"/>
-      <c r="E127" s="31"/>
-      <c r="F127" s="31"/>
-      <c r="G127" s="31"/>
-    </row>
-    <row r="128" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B127" s="42"/>
+      <c r="C127" s="42"/>
+      <c r="D127" s="42"/>
+      <c r="E127" s="42"/>
+      <c r="F127" s="42"/>
+      <c r="G127" s="42"/>
+    </row>
+    <row r="128" spans="1:7" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="14" t="s">
         <v>122</v>
       </c>
@@ -4704,10 +4409,10 @@
       <c r="E128" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="F128" s="48" t="s">
+      <c r="F128" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="G128" s="49"/>
+      <c r="G128" s="31"/>
     </row>
     <row r="129" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
@@ -4729,11 +4434,11 @@
         <f t="shared" ref="E129:E140" si="25">IF((B129+C129)=0,"",B129/(B129+C129))</f>
         <v>0.5</v>
       </c>
-      <c r="F129" s="46" t="str">
+      <c r="F129" s="28" t="str">
         <f>IF(COUNTIF(G11:G20,"INCOMPLETE")+COUNTIF(G11:G20,"MULTI")=0, "", COUNTIF(G11:G20,"INCOMPLETE")+COUNTIF(G11:G20,"MULTI") &amp; " incomplete inspection items")</f>
         <v>2 incomplete inspection items</v>
       </c>
-      <c r="G129" s="47"/>
+      <c r="G129" s="29"/>
     </row>
     <row r="130" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A130" s="5" t="s">
@@ -4755,11 +4460,11 @@
         <f t="shared" si="25"/>
         <v>0.6</v>
       </c>
-      <c r="F130" s="46" t="str">
+      <c r="F130" s="28" t="str">
         <f>IF(COUNTIF(G23:G27,"INCOMPLETE")+COUNTIF(G23:G27,"MULTI")=0, "", COUNTIF(G23:G27,"INCOMPLETE")+COUNTIF(G23:G27,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G130" s="47"/>
+      <c r="G130" s="29"/>
     </row>
     <row r="131" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A131" s="5" t="s">
@@ -4781,11 +4486,11 @@
         <f t="shared" si="25"/>
         <v>0.5714285714285714</v>
       </c>
-      <c r="F131" s="46" t="str">
+      <c r="F131" s="28" t="str">
         <f>IF(COUNTIF(G30:G37,"INCOMPLETE")+COUNTIF(G30:G37,"MULTI")=0, "", COUNTIF(G30:G37,"INCOMPLETE")+COUNTIF(G30:G37,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G131" s="47"/>
+      <c r="G131" s="29"/>
     </row>
     <row r="132" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A132" s="5" t="s">
@@ -4807,11 +4512,11 @@
         <f t="shared" si="25"/>
         <v>0.77777777777777779</v>
       </c>
-      <c r="F132" s="46" t="str">
+      <c r="F132" s="28" t="str">
         <f>IF(COUNTIF(G40:G49,"INCOMPLETE")+COUNTIF(G40:G49,"MULTI")=0, "", COUNTIF(G40:G49,"INCOMPLETE")+COUNTIF(G40:G49,"MULTI") &amp; " incomplete inspection items")</f>
         <v>1 incomplete inspection items</v>
       </c>
-      <c r="G132" s="47"/>
+      <c r="G132" s="29"/>
     </row>
     <row r="133" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A133" s="5" t="s">
@@ -4833,11 +4538,11 @@
         <f t="shared" si="25"/>
         <v>0.7</v>
       </c>
-      <c r="F133" s="46" t="str">
+      <c r="F133" s="28" t="str">
         <f>IF(COUNTIF(G52:G63,"INCOMPLETE")+COUNTIF(G52:G63,"MULTI")=0, "", COUNTIF(G52:G63,"INCOMPLETE")+COUNTIF(G52:G63,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G133" s="47"/>
+      <c r="G133" s="29"/>
     </row>
     <row r="134" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A134" s="5" t="s">
@@ -4859,11 +4564,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F134" s="46" t="str">
+      <c r="F134" s="28" t="str">
         <f>IF(COUNTIF(G66:G73,"INCOMPLETE")+COUNTIF(G66:G73,"MULTI")=0, "", COUNTIF(G66:G73,"INCOMPLETE")+COUNTIF(G66:G73,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G134" s="47"/>
+      <c r="G134" s="29"/>
     </row>
     <row r="135" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A135" s="5" t="s">
@@ -4885,11 +4590,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F135" s="46" t="str">
+      <c r="F135" s="28" t="str">
         <f>IF(COUNTIF(G76:G81,"INCOMPLETE")+COUNTIF(G76:G81,"MULTI")=0, "", COUNTIF(G76:G81,"INCOMPLETE")+COUNTIF(G76:G81,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G135" s="47"/>
+      <c r="G135" s="29"/>
     </row>
     <row r="136" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" s="5" t="s">
@@ -4911,11 +4616,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F136" s="46" t="str">
+      <c r="F136" s="28" t="str">
         <f>IF(COUNTIF(G84:G89,"INCOMPLETE")+COUNTIF(G84:G89,"MULTI")=0, "", COUNTIF(G84:G89,"INCOMPLETE")+COUNTIF(G84:G89,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G136" s="47"/>
+      <c r="G136" s="29"/>
     </row>
     <row r="137" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A137" s="5" t="s">
@@ -4937,11 +4642,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F137" s="46" t="str">
+      <c r="F137" s="28" t="str">
         <f>IF(COUNTIF(G92:G100,"INCOMPLETE")+COUNTIF(G92:G100,"MULTI")=0, "", COUNTIF(G92:G100,"INCOMPLETE")+COUNTIF(G92:G100,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G137" s="47"/>
+      <c r="G137" s="29"/>
     </row>
     <row r="138" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A138" s="5" t="s">
@@ -4963,11 +4668,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F138" s="46" t="str">
+      <c r="F138" s="28" t="str">
         <f>IF(COUNTIF(G103:G108,"INCOMPLETE")+COUNTIF(G103:G108,"MULTI")=0, "", COUNTIF(G103:G108,"INCOMPLETE")+COUNTIF(G103:G108,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G138" s="47"/>
+      <c r="G138" s="29"/>
     </row>
     <row r="139" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A139" s="5" t="s">
@@ -4989,11 +4694,11 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F139" s="46" t="str">
+      <c r="F139" s="28" t="str">
         <f>IF(COUNTIF(G111:G117,"INCOMPLETE")+COUNTIF(G111:G117,"MULTI")=0, "", COUNTIF(G111:G117,"INCOMPLETE")+COUNTIF(G111:G117,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G139" s="47"/>
+      <c r="G139" s="29"/>
     </row>
     <row r="140" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" s="5" t="s">
@@ -5015,79 +4720,104 @@
         <f t="shared" si="25"/>
         <v>1</v>
       </c>
-      <c r="F140" s="46" t="str">
+      <c r="F140" s="28" t="str">
         <f>IF(COUNTIF(G120:G124,"INCOMPLETE")+COUNTIF(G120:G124,"MULTI")=0, "", COUNTIF(G120:G124,"INCOMPLETE")+COUNTIF(G120:G124,"MULTI") &amp; " incomplete inspection items")</f>
         <v/>
       </c>
-      <c r="G140" s="47"/>
+      <c r="G140" s="29"/>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A142" s="28" t="s">
+      <c r="A142" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="B142" s="29"/>
-      <c r="C142" s="29"/>
-      <c r="D142" s="29"/>
-      <c r="E142" s="29"/>
-      <c r="F142" s="29"/>
-      <c r="G142" s="30"/>
-    </row>
-    <row r="143" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="25"/>
-      <c r="B143" s="26"/>
-      <c r="C143" s="26"/>
-      <c r="D143" s="26"/>
-      <c r="E143" s="26"/>
-      <c r="F143" s="26"/>
-      <c r="G143" s="27"/>
-    </row>
-    <row r="144" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="25"/>
-      <c r="B144" s="26"/>
-      <c r="C144" s="26"/>
-      <c r="D144" s="26"/>
-      <c r="E144" s="26"/>
-      <c r="F144" s="26"/>
-      <c r="G144" s="27"/>
-    </row>
-    <row r="145" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="25"/>
-      <c r="B145" s="26"/>
-      <c r="C145" s="26"/>
-      <c r="D145" s="26"/>
-      <c r="E145" s="26"/>
-      <c r="F145" s="26"/>
-      <c r="G145" s="27"/>
-    </row>
-    <row r="146" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="25"/>
-      <c r="B146" s="26"/>
-      <c r="C146" s="26"/>
-      <c r="D146" s="26"/>
-      <c r="E146" s="26"/>
-      <c r="F146" s="26"/>
-      <c r="G146" s="27"/>
-    </row>
-    <row r="147" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="25"/>
-      <c r="B147" s="26"/>
-      <c r="C147" s="26"/>
-      <c r="D147" s="26"/>
-      <c r="E147" s="26"/>
-      <c r="F147" s="26"/>
-      <c r="G147" s="27"/>
-    </row>
-    <row r="148" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="25"/>
-      <c r="B148" s="26"/>
-      <c r="C148" s="26"/>
-      <c r="D148" s="26"/>
-      <c r="E148" s="26"/>
-      <c r="F148" s="26"/>
-      <c r="G148" s="27"/>
+      <c r="B142" s="51"/>
+      <c r="C142" s="51"/>
+      <c r="D142" s="51"/>
+      <c r="E142" s="51"/>
+      <c r="F142" s="51"/>
+      <c r="G142" s="52"/>
+    </row>
+    <row r="143" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="47"/>
+      <c r="B143" s="48"/>
+      <c r="C143" s="48"/>
+      <c r="D143" s="48"/>
+      <c r="E143" s="48"/>
+      <c r="F143" s="48"/>
+      <c r="G143" s="49"/>
+    </row>
+    <row r="144" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="47"/>
+      <c r="B144" s="48"/>
+      <c r="C144" s="48"/>
+      <c r="D144" s="48"/>
+      <c r="E144" s="48"/>
+      <c r="F144" s="48"/>
+      <c r="G144" s="49"/>
+    </row>
+    <row r="145" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="47"/>
+      <c r="B145" s="48"/>
+      <c r="C145" s="48"/>
+      <c r="D145" s="48"/>
+      <c r="E145" s="48"/>
+      <c r="F145" s="48"/>
+      <c r="G145" s="49"/>
+    </row>
+    <row r="146" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="47"/>
+      <c r="B146" s="48"/>
+      <c r="C146" s="48"/>
+      <c r="D146" s="48"/>
+      <c r="E146" s="48"/>
+      <c r="F146" s="48"/>
+      <c r="G146" s="49"/>
+    </row>
+    <row r="147" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="47"/>
+      <c r="B147" s="48"/>
+      <c r="C147" s="48"/>
+      <c r="D147" s="48"/>
+      <c r="E147" s="48"/>
+      <c r="F147" s="48"/>
+      <c r="G147" s="49"/>
+    </row>
+    <row r="148" spans="1:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="47"/>
+      <c r="B148" s="48"/>
+      <c r="C148" s="48"/>
+      <c r="D148" s="48"/>
+      <c r="E148" s="48"/>
+      <c r="F148" s="48"/>
+      <c r="G148" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="A148:G148"/>
+    <mergeCell ref="A142:G142"/>
+    <mergeCell ref="A143:G143"/>
+    <mergeCell ref="A144:G144"/>
+    <mergeCell ref="A145:G145"/>
+    <mergeCell ref="A146:G146"/>
+    <mergeCell ref="A147:G147"/>
+    <mergeCell ref="A127:G127"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A65:G65"/>
+    <mergeCell ref="A75:G75"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A91:G91"/>
+    <mergeCell ref="A102:G102"/>
+    <mergeCell ref="A110:G110"/>
+    <mergeCell ref="A119:G119"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="F139:G139"/>
     <mergeCell ref="F140:G140"/>
     <mergeCell ref="F128:G128"/>
@@ -5101,31 +4831,6 @@
     <mergeCell ref="F131:G131"/>
     <mergeCell ref="F132:G132"/>
     <mergeCell ref="F133:G133"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A127:G127"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="A65:G65"/>
-    <mergeCell ref="A75:G75"/>
-    <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A91:G91"/>
-    <mergeCell ref="A102:G102"/>
-    <mergeCell ref="A110:G110"/>
-    <mergeCell ref="A119:G119"/>
-    <mergeCell ref="A148:G148"/>
-    <mergeCell ref="A142:G142"/>
-    <mergeCell ref="A143:G143"/>
-    <mergeCell ref="A144:G144"/>
-    <mergeCell ref="A145:G145"/>
-    <mergeCell ref="A146:G146"/>
-    <mergeCell ref="A147:G147"/>
   </mergeCells>
   <conditionalFormatting sqref="A56">
     <cfRule type="expression" dxfId="134" priority="275">
@@ -5173,11 +4878,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A84:B89">
-    <cfRule type="expression" dxfId="123" priority="178">
+    <cfRule type="expression" dxfId="123" priority="180">
+      <formula>$G84="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="122" priority="178">
       <formula>$C84="X"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="122" priority="180">
-      <formula>$G84="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A111:B117">
@@ -5197,11 +4902,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11:C20">
-    <cfRule type="expression" dxfId="117" priority="148">
+    <cfRule type="expression" dxfId="117" priority="149">
+      <formula>$G11="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="116" priority="148">
       <formula>$C11="X"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="116" priority="149">
-      <formula>$G11="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
@@ -5220,14 +4925,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B37">
-    <cfRule type="expression" dxfId="112" priority="208">
-      <formula>$C30="X"</formula>
+    <cfRule type="expression" dxfId="112" priority="210">
+      <formula>$G30="MULTI"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="111" priority="209">
       <formula>$B30="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="110" priority="210">
-      <formula>$G30="MULTI"</formula>
+    <cfRule type="expression" dxfId="110" priority="208">
+      <formula>$C30="X"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B40:B49">
@@ -5251,11 +4956,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92:B100">
-    <cfRule type="expression" dxfId="105" priority="175">
+    <cfRule type="expression" dxfId="105" priority="177">
+      <formula>$G92="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="104" priority="175">
       <formula>$C92="X"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="104" priority="177">
-      <formula>$G92="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92:B101">
@@ -5332,14 +5037,14 @@
     <cfRule type="expression" dxfId="87" priority="144">
       <formula>$B31="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="86" priority="143">
-      <formula>$G31="MULTI"</formula>
+    <cfRule type="expression" dxfId="86" priority="141">
+      <formula>$C31="X"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="85" priority="142">
       <formula>$B31="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="141">
-      <formula>$C31="X"</formula>
+    <cfRule type="expression" dxfId="84" priority="143">
+      <formula>$G31="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C36:C37">
@@ -5357,22 +5062,22 @@
     <cfRule type="expression" dxfId="80" priority="138">
       <formula>$C47="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="79" priority="140">
+    <cfRule type="expression" dxfId="79" priority="139">
+      <formula>$B47="X"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="78" priority="140">
       <formula>$G47="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="139">
-      <formula>$B47="X"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C77:C78">
-    <cfRule type="expression" dxfId="77" priority="193">
-      <formula>$C77="X"</formula>
+    <cfRule type="expression" dxfId="77" priority="194">
+      <formula>$B77="X"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="76" priority="195">
       <formula>$G77="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="194">
-      <formula>$B77="X"</formula>
+    <cfRule type="expression" dxfId="75" priority="193">
+      <formula>$C77="X"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23:E23 D24:E25 C26:E27">
@@ -5466,19 +5171,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:G37">
-    <cfRule type="expression" dxfId="56" priority="46">
+    <cfRule type="expression" dxfId="56" priority="45">
+      <formula>$C30="X"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="46">
       <formula>$G30="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="45">
-      <formula>$C30="X"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F40:G49">
-    <cfRule type="expression" dxfId="54" priority="41">
+    <cfRule type="expression" dxfId="54" priority="40">
+      <formula>$C40="X"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="53" priority="41">
       <formula>$G40="MULTI"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="53" priority="40">
-      <formula>$C40="X"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F66:G73">
@@ -5498,74 +5203,74 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F84:G89">
-    <cfRule type="expression" dxfId="48" priority="23">
+    <cfRule type="expression" dxfId="48" priority="22">
+      <formula>$C84="X"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="47" priority="23">
       <formula>$G84="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="22">
-      <formula>$C84="X"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F92:G100">
-    <cfRule type="expression" dxfId="46" priority="18">
+    <cfRule type="expression" dxfId="46" priority="17">
+      <formula>$C92="X"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="18">
       <formula>$G92="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="17">
-      <formula>$C92="X"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F111:G117">
-    <cfRule type="expression" dxfId="44" priority="9">
+    <cfRule type="expression" dxfId="44" priority="10">
+      <formula>$G111="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="9">
       <formula>$C111="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="10">
-      <formula>$G111="MULTI"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F120:G124">
-    <cfRule type="expression" dxfId="42" priority="4">
+    <cfRule type="expression" dxfId="42" priority="5">
+      <formula>$G120="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="4">
       <formula>$C120="X"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="5">
-      <formula>$G120="MULTI"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G20">
-    <cfRule type="expression" dxfId="40" priority="105">
-      <formula>$G11="MULTI"</formula>
+    <cfRule type="expression" dxfId="40" priority="107">
+      <formula>$G11="Incomplete"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="39" priority="106">
       <formula>$G11="COMPLETE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="107">
-      <formula>$G11="Incomplete"</formula>
+    <cfRule type="expression" dxfId="38" priority="105">
+      <formula>$G11="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G23:G27">
     <cfRule type="expression" dxfId="37" priority="49">
       <formula>$G23="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="47">
+    <cfRule type="expression" dxfId="36" priority="101">
       <formula>$G23="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="48">
+    <cfRule type="expression" dxfId="35" priority="102">
       <formula>$G23="COMPLETE"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="34" priority="103">
       <formula>$G23="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="102">
+    <cfRule type="expression" dxfId="33" priority="48">
       <formula>$G23="COMPLETE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="101">
+    <cfRule type="expression" dxfId="32" priority="47">
       <formula>$G23="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G37">
-    <cfRule type="expression" dxfId="31" priority="43">
+    <cfRule type="expression" dxfId="31" priority="44">
+      <formula>$G30="Incomplete"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="30" priority="43">
       <formula>$G30="COMPLETE"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="30" priority="44">
-      <formula>$G30="Incomplete"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="29" priority="42">
       <formula>$G30="MULTI"</formula>
@@ -5586,44 +5291,44 @@
     <cfRule type="expression" dxfId="25" priority="36">
       <formula>$G52="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="35">
+    <cfRule type="expression" dxfId="24" priority="34">
+      <formula>$G52="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="35">
       <formula>$G52="COMPLETE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="34">
-      <formula>$G52="MULTI"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G66:G73">
-    <cfRule type="expression" dxfId="22" priority="31">
-      <formula>$G66="Incomplete"</formula>
+    <cfRule type="expression" dxfId="22" priority="29">
+      <formula>$G66="MULTI"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="21" priority="30">
       <formula>$G66="COMPLETE"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="29">
-      <formula>$G66="MULTI"</formula>
+    <cfRule type="expression" dxfId="20" priority="31">
+      <formula>$G66="Incomplete"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G76:G81">
-    <cfRule type="expression" dxfId="19" priority="26">
+    <cfRule type="expression" dxfId="19" priority="24">
+      <formula>$G76="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="25">
+      <formula>$G76="COMPLETE"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="26">
       <formula>$G76="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="24">
-      <formula>$G76="MULTI"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="25">
-      <formula>$G76="COMPLETE"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G84:G89">
-    <cfRule type="expression" dxfId="16" priority="20">
-      <formula>$G84="COMPLETE"</formula>
+    <cfRule type="expression" dxfId="16" priority="19">
+      <formula>$G84="MULTI"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="15" priority="21">
       <formula>$G84="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="19">
-      <formula>$G84="MULTI"</formula>
+    <cfRule type="expression" dxfId="14" priority="20">
+      <formula>$G84="COMPLETE"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G92:G100">
@@ -5638,11 +5343,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G103:G108">
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>$G103="MULTI"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="12">
       <formula>$G103="COMPLETE"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="11">
-      <formula>$G103="MULTI"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="8" priority="13">
       <formula>$G103="Incomplete"</formula>
@@ -5652,40 +5357,47 @@
     <cfRule type="expression" dxfId="7" priority="6">
       <formula>$G111="MULTI"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="6" priority="7">
+      <formula>$G111="COMPLETE"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>$G111="Incomplete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="7">
-      <formula>$G111="COMPLETE"</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G120:G124">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="4" priority="3">
+      <formula>$G120="Incomplete"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$G120="COMPLETE"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$G120="Incomplete"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>$G120="MULTI"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="B92:D101 B23:D27 B111:D117 B40:D49 B11:D21 B76:D81 B66:D73 B120:D124 B84:D89 B103:D108 B30:D37 B52:D63" xr:uid="{86737741-0F17-4FC2-B5FC-6A3A5385C2EC}">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="B92:D101 B23:D27 B111:D117 B40:D49 B11:D21 B76:D81 B66:D73 B120:D124 B84:D89 B103:D108 B30:D37 B52:D63" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>" ,X"</formula1>
     </dataValidation>
+    <dataValidation type="date" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid inspection date" error="Enter a valid calendar date." promptTitle="Inspection date" prompt="Enter the inspection date used for the weekly reporting period." sqref="B3" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>DATE(2000,1,1)</formula1>
+      <formula2>DATE(2100,12,31)</formula2>
+    </dataValidation>
+    <dataValidation type="whole" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid inspection number" error="Enter a whole number." promptTitle="Inspection number" prompt="Enter a whole-number inspection sequence value." sqref="E3" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>0</formula1>
+      <formula2>1000000</formula2>
+    </dataValidation>
   </dataValidations>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="73" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC020783-A7D5-4D0E-BEFD-8C60B53DDE83}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="23.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.5" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
@@ -5879,11 +5591,11 @@
         <v>141</v>
       </c>
       <c r="C14" s="22">
-        <f>SUM(tblWeights[Weight])</f>
+        <f ca="1">SUM(tblWeights[Weight])</f>
         <v>1.0000000000000002</v>
       </c>
       <c r="D14" s="23" t="str">
-        <f>IF(ABS(1-SUM(tblWeights[Weight]))&lt;=0.000001,"",IF(1-SUM(tblWeights[Weight])&gt;0,"Add "&amp;TEXT(1-SUM(tblWeights[Weight]),"0%")&amp;" to the category weights","Deduct "&amp;TEXT(ABS(1-SUM(tblWeights[Weight])),"0%")&amp;" from the category weights"))</f>
+        <f ca="1">IF(ABS(1-SUM(tblWeights[Weight]))&lt;=0.000001,"",IF(1-SUM(tblWeights[Weight])&gt;0,"Add "&amp;TEXT(1-SUM(tblWeights[Weight]),"0%")&amp;" to the category weights","Deduct "&amp;TEXT(ABS(1-SUM(tblWeights[Weight])),"0%")&amp;" from the category weights"))</f>
         <v/>
       </c>
     </row>
@@ -5901,4 +5613,184 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B4" s="25">
+        <f>ScoreCard!B3</f>
+        <v>46068</v>
+      </c>
+      <c r="C4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B5">
+        <f>ScoreCard!E3</f>
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6">
+        <f>ScoreCard!B4</f>
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7">
+        <f>ScoreCard!G4</f>
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8">
+        <f>ScoreCard!G5</f>
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B9">
+        <f>ScoreCard!G6</f>
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="26">
+        <f>ScoreCard!G7</f>
+        <v>0.85671428571428576</v>
+      </c>
+      <c r="C10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="25">
+        <f>IF(B4="","",INT(B4))</f>
+        <v>46068</v>
+      </c>
+      <c r="C11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B12" s="25">
+        <f>IF(B11="","",B11+4)</f>
+        <v>46072</v>
+      </c>
+      <c r="C12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>169</v>
+      </c>
+      <c r="B13" s="27" t="str">
+        <f>IF(OR(B11="",B12=""),"",TEXT(B11,"mmmm d")&amp;" - "&amp;TEXT(B12,"mmmm d, yyyy"))</f>
+        <v>February 15 - February 19, 2026</v>
+      </c>
+      <c r="C13" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" t="e">
+        <f ca="1">_xludf.TEXTJOIN(CHAR(10),TRUE,ScoreCard!A143,ScoreCard!A144,ScoreCard!A145,ScoreCard!A146,ScoreCard!A147,ScoreCard!A148)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="C14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>